<commit_message>
docs(lit): add URSim and static-vs-dynamic papers from S20 research
</commit_message>
<xml_diff>
--- a/docs/literature_review.xlsx
+++ b/docs/literature_review.xlsx
@@ -615,6 +615,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
@@ -1566,70 +1568,258 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>le2025ur</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Le TD, Le M</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Empowering Universal Robot Programming with Fine-Tuned Large Language Models</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>EAI Endorsed Transactions on AI and Robotics</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>https://publications.eai.eu/index.php/airo/article/view/8983</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>10.4108/airo.8983</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>simulator_precedent</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>hu2024codebotler</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Hu Z, Lucchetti F, Schlesinger C, Saxena Y, Freeman A, Modak S, Guha A, Biswas J</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Deploying and Evaluating LLMs to Program Service Mobile Robots</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Robotics and Automation Letters</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>https://amrl.cs.utexas.edu/codebotler/</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/LRA.2024.3360020</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>llm_robot_code_ral_precedent</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>adversarial_secure_code_2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>(authors listed in arXiv record)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>How Secure is Secure Code Generation? Adversarial Prompts Put LLM Defenses to the Test</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>arXiv (preprint)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2601.07084</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>static_analyzer_threat</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>secure_code_eval_rethink_2025</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>(authors listed in arXiv record)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Rethinking the Evaluation of Secure Code Generation</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>arXiv (preprint)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2503.15554</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>secure_code_eval_methodology</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>roboguard_2025</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>(authors anonymized OpenReview)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Safety Guardrails for LLM-Enabled Robots (ROBOGUARD)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>OpenReview preprint (venue TBD)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>https://openreview.net/pdf/266d74ff750008c876587179f313b5981f5400ee.pdf</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>llm_robot_safety_formal</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>reachability_llm_safety_2025</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>(authors listed in arXiv record)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Safe LLM-Controlled Robots with Formal Guarantees via Reachability Analysis</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>arXiv (preprint)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2503.03911</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>llm_robot_safety_formal</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -4575,64 +4765,256 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>G023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>le2025ur</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Uses URSim 5.12.6 LTS for LLM-generated URScript evaluation but has no adversarial or security focus; fine-tuning accuracy only.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>[paraphrase] Uses URSim offline simulator for UR3 fine-tuning data</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Methods; Reference [13] URSim 5.12.6 LTS</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Only known academic precedent for URSim as LLM URScript evaluation simulator. Justifies ENFIELD simulator choice against 'niche tool' critique. Lower-tier venue (EAI) but scopus-indexed.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>methodology</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>strengthens_us</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>G024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>hu2024codebotler</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>RA-L precedent for LLM-generated robot code evaluation; uses symbolic simulator + temporal-logic trace check, not physics simulation.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>[paraphrase] Symbolic simulator executes the program and outputs trace</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Methods section; RoboEval framework description</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Establishes RA-L venue acceptance for execution-based trace evaluation without full physics simulation. Directly supports our URSim-only scope argument for RA-L submission.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>methodology</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>strengthens_us</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>G025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>adversarial_secure_code_2026</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Static analyzers overestimate security 7 to 21x relative to execution-based oracles; under adversarial prompts secure-and-functional rate collapses to 3-17%.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>static analyzers overestimate security by 7 to 21 times</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Direct reviewer threat: ENFIELD SM-1..7 are static analyzers on URScript AST. Must preemptively address in §VII.B. Domain narrowness (URScript) and deterministic AST mitigate but do not eliminate this critique.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>H4, H5, H6</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>threatens_us</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>G026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>secure_code_eval_rethink_2025</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Secure-code techniques often remove vulnerable lines entirely or generate garbage code unrelated to task; technique performance degrades base LLM.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>[paraphrase] Techniques remove vulnerable lines or generate garbage code</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Abstract; Introduction</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Directly echoes ENFIELD §VI.H watchdog-via-invalidation artefact (DeepSeek baseline 44% gate-pass drops to 4% under watchdog-in-loop). External literature support for honest framing of H6 mechanism.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>G027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>roboguard_2025</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>LLM robot guardrail using LTL safety specs + control synthesis + Buchi automata; evaluated in simulation and on real Clearpath Jackal.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>[paraphrase] LTL-based root-of-trust LLM with controller synthesis</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Abstract; Algorithm 1</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Alternative paradigm (formal methods + simulation) to ENFIELD's static AST watchdog. Not direct competitor but establishes that LLM robot safety is actively researched with execution-based validation.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>G028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>reachability_llm_safety_2025</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Formal safety assurance via data-driven reachability analysis layered on top of LLM-generated plans; collision-free guarantees with failsafe.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>[paraphrase] Data-driven reachability-based safety filter on LLM plans</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Abstract; Algorithm 1</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Another alternative paradigm using formal verification. Like RoboGuard, assumes execution-time intervention rather than static pre-execution analysis. Positions ENFIELD as static-analysis complement not replacement.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>

</xml_diff>